<commit_message>
some updates:delete unused files and update data with real nip data
</commit_message>
<xml_diff>
--- a/public/asset/template_guru.xlsx
+++ b/public/asset/template_guru.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\SIMPEL-5\public\asset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B375FEE-2820-43C6-8DAF-CE7B42408268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6F1ACC-9A15-4841-8634-DC4226196F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B5C1236F-2DC1-4DEB-9CB8-AC0626038A09}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>nama</t>
   </si>
@@ -48,92 +48,71 @@
     <t>nip</t>
   </si>
   <si>
-    <t>Lidia Arlini</t>
-  </si>
-  <si>
-    <t>Teknik Komputer dan Jaringan</t>
-  </si>
-  <si>
-    <t>Muthia Wiyaningsih</t>
-  </si>
-  <si>
     <t>Rekayasa Perangkat Lunak</t>
   </si>
   <si>
-    <t>Eko Ayatullah</t>
-  </si>
-  <si>
     <t>Teknik Kendaraan Ringan</t>
   </si>
   <si>
-    <t>Maylan Syabani</t>
-  </si>
-  <si>
-    <t>Teknik Sepeda Motor</t>
-  </si>
-  <si>
     <t>Armansyah</t>
   </si>
   <si>
     <t>Teknik Permesinan</t>
   </si>
   <si>
-    <t>Tati Munsicha</t>
-  </si>
-  <si>
     <t>Manajemen Perkantoran</t>
   </si>
   <si>
-    <t>Randy Himaktiar</t>
-  </si>
-  <si>
-    <t>Akuntansi Keuangan Lembaga</t>
-  </si>
-  <si>
-    <t>Saleha</t>
-  </si>
-  <si>
-    <t>Mukti Prasetyo</t>
-  </si>
-  <si>
-    <t>Perhotelan</t>
-  </si>
-  <si>
-    <t>Agribisnis Pengolahan Hasil Perikanan</t>
-  </si>
-  <si>
-    <t>lidia@gmail.com</t>
-  </si>
-  <si>
     <t>muthia@gmail.com</t>
   </si>
   <si>
     <t>eko@gmail.com</t>
   </si>
   <si>
-    <t>maylan@gmail.com</t>
-  </si>
-  <si>
     <t>armansyah@gmail.com</t>
   </si>
   <si>
     <t>tati@gmail.com</t>
   </si>
   <si>
-    <t>randy@gmail.com</t>
-  </si>
-  <si>
-    <t>saleha@gmail.com</t>
-  </si>
-  <si>
-    <t>mukti@gmail.com</t>
+    <t>Muthia Widyaningsih</t>
+  </si>
+  <si>
+    <t>Adam Kurniahan Susanto</t>
+  </si>
+  <si>
+    <t>198703172025211000</t>
+  </si>
+  <si>
+    <t>198109122010012007</t>
+  </si>
+  <si>
+    <t>198001512021212012</t>
+  </si>
+  <si>
+    <t>Tati Munsicha, S.Pd.</t>
+  </si>
+  <si>
+    <t>Eko Ayatullah Khomaeini</t>
+  </si>
+  <si>
+    <t>198104072022211000</t>
+  </si>
+  <si>
+    <t>198412012022211000</t>
+  </si>
+  <si>
+    <t>Desain Komunikasi Visual</t>
+  </si>
+  <si>
+    <t>adam@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,6 +148,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -191,18 +176,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -518,17 +500,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFAD8768-4066-4A27-B449-170C24190DD5}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.54296875" customWidth="1"/>
-    <col min="2" max="2" width="17.90625" customWidth="1"/>
+    <col min="2" max="2" width="20.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.453125" customWidth="1"/>
     <col min="4" max="4" width="27.6328125" customWidth="1"/>
     <col min="5" max="5" width="8.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -542,153 +524,103 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
-        <v>19800102</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="D5" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
-        <v>19800103</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2">
-        <v>19800104</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2">
-        <v>19800105</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="4"/>
-    </row>
-    <row r="6" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="2">
-        <v>19800106</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="4"/>
-    </row>
-    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="2">
-        <v>19800107</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="4"/>
-    </row>
-    <row r="8" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2">
-        <v>19800108</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="4"/>
-    </row>
-    <row r="9" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="2">
-        <v>19800109</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="4"/>
-    </row>
-    <row r="10" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="2">
-        <v>19800110</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{2364BFCB-586E-459A-A859-134981AAC12A}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{D8911725-4DB5-40CA-B24E-118B5D076BBB}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{DD4B05A9-E738-4563-ACC3-2F74373F5D98}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{53BC5A73-437B-4A72-883D-03569237459C}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{A1914D54-285B-44F9-ABAB-8522875334E4}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{6E382DA7-A4FE-4B85-B6BC-318817CF0D89}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{78AA78A1-4482-46BA-9645-A7D7962FFE56}"/>
-    <hyperlink ref="D9" r:id="rId8" xr:uid="{D5378526-E007-4855-9779-2867F563813A}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{EE08C4C0-C85A-4B28-B58A-9ACAA863B272}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{6B5D1A8C-1A56-4283-98B4-5C55CA1F0239}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{F2B57BA4-8C08-425F-8035-AE5028A51A5E}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{E25FF966-C454-44BB-A506-49B45DBC1030}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{742503C5-812D-43EA-B268-E5A3D7C6674A}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{9FDD9722-E5FC-4D22-AEB4-281CDC28EA4C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+  <ignoredErrors>
+    <ignoredError sqref="B3:B6" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>